<commit_message>
Update analyst ratings and add LAPWALL to targets list
</commit_message>
<xml_diff>
--- a/Manual_Analyst_Ratings.xlsx
+++ b/Manual_Analyst_Ratings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/casperkangas/Documents/VS Code/Personal Projects/nordnet-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB4854C1-2C1D-BE4A-AA86-2D5855E81685}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F741D978-F166-3E46-9F53-0464244FDDCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="18000" yWindow="780" windowWidth="18000" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="124">
   <si>
     <t>Ticker</t>
   </si>
@@ -405,6 +405,9 @@
   </si>
   <si>
     <t>IQMX</t>
+  </si>
+  <si>
+    <t>LAPWALL</t>
   </si>
 </sst>
 </file>
@@ -776,7 +779,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1971DA79-8A22-7244-902F-F8980870F481}">
-  <dimension ref="A1:G117"/>
+  <dimension ref="A1:G118"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -807,22 +810,22 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2">
         <v>5</v>
       </c>
       <c r="E2">
-        <v>-23.93</v>
+        <v>-21.7</v>
       </c>
       <c r="F2">
-        <v>3.6</v>
+        <v>2.91</v>
       </c>
       <c r="G2">
-        <v>14.11</v>
+        <v>15.21</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -839,13 +842,13 @@
         <v>2</v>
       </c>
       <c r="E3">
-        <v>-14.77</v>
+        <v>-12.02</v>
       </c>
       <c r="F3">
-        <v>12.97</v>
+        <v>16.62</v>
       </c>
       <c r="G3">
-        <v>65.72</v>
+        <v>71.069999999999993</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -853,7 +856,7 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C4">
         <v>6</v>
@@ -862,13 +865,13 @@
         <v>7</v>
       </c>
       <c r="E4">
-        <v>-46.72</v>
+        <v>-49.35</v>
       </c>
       <c r="F4">
-        <v>26.03</v>
+        <v>20.37</v>
       </c>
       <c r="G4">
-        <v>106.23</v>
+        <v>96.08</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -885,13 +888,13 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>-2.16</v>
+        <v>-2.46</v>
       </c>
       <c r="F5">
-        <v>0.69</v>
+        <v>0.38</v>
       </c>
       <c r="G5">
-        <v>4.01</v>
+        <v>3.69</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -908,13 +911,13 @@
         <v>5</v>
       </c>
       <c r="E6">
-        <v>-21.26</v>
+        <v>-20.51</v>
       </c>
       <c r="F6">
-        <v>-3.62</v>
+        <v>-2.7</v>
       </c>
       <c r="G6">
-        <v>10.24</v>
+        <v>11.29</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -931,7 +934,7 @@
         <v>1</v>
       </c>
       <c r="F7">
-        <v>0.24</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -948,13 +951,13 @@
         <v>1</v>
       </c>
       <c r="E8">
-        <v>-38.79</v>
+        <v>-37</v>
       </c>
       <c r="F8">
-        <v>-5.87</v>
+        <v>-3.12</v>
       </c>
       <c r="G8">
-        <v>11.3</v>
+        <v>14.55</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -971,7 +974,7 @@
         <v>0</v>
       </c>
       <c r="F9">
-        <v>6.38</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -985,16 +988,16 @@
         <v>8</v>
       </c>
       <c r="D10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10">
-        <v>-31.88</v>
+        <v>-34.75</v>
       </c>
       <c r="F10">
-        <v>20.04</v>
+        <v>14.87</v>
       </c>
       <c r="G10">
-        <v>54.18</v>
+        <v>47.55</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -1011,13 +1014,13 @@
         <v>1</v>
       </c>
       <c r="E11">
-        <v>-14.74</v>
+        <v>-11.63</v>
       </c>
       <c r="F11">
-        <v>16.14</v>
+        <v>20.38</v>
       </c>
       <c r="G11">
-        <v>57.26</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -1034,13 +1037,13 @@
         <v>3</v>
       </c>
       <c r="E12">
-        <v>-24.2</v>
+        <v>-25.62</v>
       </c>
       <c r="F12">
-        <v>0.56000000000000005</v>
+        <v>-1.32</v>
       </c>
       <c r="G12">
-        <v>20.72</v>
+        <v>18.46</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -1048,22 +1051,22 @@
         <v>18</v>
       </c>
       <c r="B13">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C13">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E13">
-        <v>-42.28</v>
+        <v>-43.7</v>
       </c>
       <c r="F13">
-        <v>6.15</v>
+        <v>6.33</v>
       </c>
       <c r="G13">
-        <v>66.25</v>
+        <v>62.18</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -1080,13 +1083,13 @@
         <v>12</v>
       </c>
       <c r="E14">
-        <v>-29.54</v>
+        <v>-31.16</v>
       </c>
       <c r="F14">
-        <v>-12.11</v>
+        <v>-14.14</v>
       </c>
       <c r="G14">
-        <v>6.18</v>
+        <v>3.72</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -1103,13 +1106,13 @@
         <v>0</v>
       </c>
       <c r="E15">
-        <v>20.03</v>
+        <v>25.43</v>
       </c>
       <c r="F15">
-        <v>28.31</v>
+        <v>34.08</v>
       </c>
       <c r="G15">
-        <v>36.590000000000003</v>
+        <v>42.73</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -1126,13 +1129,13 @@
         <v>0</v>
       </c>
       <c r="E16">
-        <v>-2.2200000000000002</v>
+        <v>-1.1599999999999999</v>
       </c>
       <c r="F16">
-        <v>8.3699999999999992</v>
+        <v>9.44</v>
       </c>
       <c r="G16">
-        <v>15.16</v>
+        <v>16.399999999999999</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
@@ -1149,13 +1152,13 @@
         <v>5</v>
       </c>
       <c r="E17">
-        <v>-27.68</v>
+        <v>-27.86</v>
       </c>
       <c r="F17">
-        <v>7.86</v>
+        <v>7.59</v>
       </c>
       <c r="G17">
-        <v>57.94</v>
+        <v>57.55</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
@@ -1172,13 +1175,13 @@
         <v>2</v>
       </c>
       <c r="E18">
-        <v>-20.99</v>
+        <v>-21.38</v>
       </c>
       <c r="F18">
-        <v>10.42</v>
+        <v>9.8800000000000008</v>
       </c>
       <c r="G18">
-        <v>33.33</v>
+        <v>32.68</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
@@ -1195,13 +1198,13 @@
         <v>2</v>
       </c>
       <c r="E19">
-        <v>-30.47</v>
+        <v>-30.82</v>
       </c>
       <c r="F19">
-        <v>-2.11</v>
+        <v>-2.6</v>
       </c>
       <c r="G19">
-        <v>8.7200000000000006</v>
+        <v>8.18</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
@@ -1218,13 +1221,13 @@
         <v>2</v>
       </c>
       <c r="E20">
-        <v>-2.96</v>
+        <v>4.05</v>
       </c>
       <c r="F20">
-        <v>6.25</v>
+        <v>13.93</v>
       </c>
       <c r="G20">
-        <v>15.9</v>
+        <v>24.28</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -1232,22 +1235,22 @@
         <v>26</v>
       </c>
       <c r="B21">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C21">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D21">
         <v>4</v>
       </c>
       <c r="E21">
-        <v>-5.01</v>
+        <v>-5.86</v>
       </c>
       <c r="F21">
-        <v>13.23</v>
+        <v>10.6</v>
       </c>
       <c r="G21">
-        <v>42.21</v>
+        <v>40.92</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -1264,13 +1267,13 @@
         <v>7</v>
       </c>
       <c r="E22">
-        <v>-29.63</v>
+        <v>-30.5</v>
       </c>
       <c r="F22">
-        <v>6.32</v>
+        <v>5</v>
       </c>
       <c r="G22">
-        <v>37.68</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
@@ -1287,13 +1290,13 @@
         <v>1</v>
       </c>
       <c r="E23">
-        <v>-20.36</v>
+        <v>-18.05</v>
       </c>
       <c r="F23">
-        <v>-3.78</v>
+        <v>-1.45</v>
       </c>
       <c r="G23">
-        <v>18.45</v>
+        <v>21.89</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
@@ -1310,13 +1313,13 @@
         <v>0</v>
       </c>
       <c r="E24">
-        <v>1.32</v>
+        <v>2.35</v>
       </c>
       <c r="F24">
-        <v>6.38</v>
+        <v>7.47</v>
       </c>
       <c r="G24">
-        <v>16.510000000000002</v>
+        <v>17.71</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
@@ -1333,13 +1336,13 @@
         <v>0</v>
       </c>
       <c r="E25">
-        <v>20.12</v>
+        <v>18.690000000000001</v>
       </c>
       <c r="F25">
-        <v>23.12</v>
+        <v>21.66</v>
       </c>
       <c r="G25">
-        <v>26.13</v>
+        <v>24.63</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
@@ -1356,7 +1359,7 @@
         <v>0</v>
       </c>
       <c r="F26">
-        <v>-16.32</v>
+        <v>-15.25</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
@@ -1373,7 +1376,7 @@
         <v>0</v>
       </c>
       <c r="F27">
-        <v>3.66</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
@@ -1390,7 +1393,7 @@
         <v>1</v>
       </c>
       <c r="F28">
-        <v>2.16</v>
+        <v>10.97</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
@@ -1421,7 +1424,7 @@
         <v>0</v>
       </c>
       <c r="F30">
-        <v>8.8699999999999992</v>
+        <v>11.11</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -1438,13 +1441,13 @@
         <v>2</v>
       </c>
       <c r="E31">
-        <v>4.8</v>
+        <v>7.14</v>
       </c>
       <c r="F31">
-        <v>6.99</v>
+        <v>9.3800000000000008</v>
       </c>
       <c r="G31">
-        <v>9.17</v>
+        <v>11.61</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
@@ -1461,13 +1464,13 @@
         <v>0</v>
       </c>
       <c r="E32">
-        <v>4.43</v>
+        <v>6.04</v>
       </c>
       <c r="F32">
-        <v>19.809999999999999</v>
+        <v>21.66</v>
       </c>
       <c r="G32">
-        <v>32.909999999999997</v>
+        <v>34.96</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
@@ -1484,7 +1487,7 @@
         <v>0</v>
       </c>
       <c r="F33">
-        <v>16.28</v>
+        <v>15.77</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
@@ -1501,13 +1504,13 @@
         <v>1</v>
       </c>
       <c r="E34">
-        <v>-0.26</v>
+        <v>-1.81</v>
       </c>
       <c r="F34">
-        <v>19.03</v>
+        <v>17.18</v>
       </c>
       <c r="G34">
-        <v>31.23</v>
+        <v>29.2</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
@@ -1524,13 +1527,13 @@
         <v>0</v>
       </c>
       <c r="E35">
-        <v>-3.31</v>
+        <v>-1.1299999999999999</v>
       </c>
       <c r="F35">
-        <v>14.36</v>
+        <v>16.95</v>
       </c>
       <c r="G35">
-        <v>28.91</v>
+        <v>31.83</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
@@ -1538,7 +1541,7 @@
         <v>41</v>
       </c>
       <c r="B36">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C36">
         <v>1</v>
@@ -1547,13 +1550,13 @@
         <v>0</v>
       </c>
       <c r="E36">
-        <v>4.42</v>
+        <v>10.6</v>
       </c>
       <c r="F36">
-        <v>19.61</v>
+        <v>27.55</v>
       </c>
       <c r="G36">
-        <v>33.869999999999997</v>
+        <v>43.05</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
@@ -1570,13 +1573,13 @@
         <v>0</v>
       </c>
       <c r="E37">
-        <v>5.78</v>
+        <v>7.78</v>
       </c>
       <c r="F37">
-        <v>7.96</v>
+        <v>10</v>
       </c>
       <c r="G37">
-        <v>9.0500000000000007</v>
+        <v>11.11</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
@@ -1593,13 +1596,13 @@
         <v>0</v>
       </c>
       <c r="E38">
-        <v>4.7300000000000004</v>
+        <v>5.01</v>
       </c>
       <c r="F38">
-        <v>17.260000000000002</v>
+        <v>17.579999999999998</v>
       </c>
       <c r="G38">
-        <v>28.38</v>
+        <v>28.73</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
@@ -1616,13 +1619,13 @@
         <v>0</v>
       </c>
       <c r="E39">
-        <v>-5.86</v>
+        <v>-5.0599999999999996</v>
       </c>
       <c r="F39">
-        <v>10.08</v>
+        <v>11.01</v>
       </c>
       <c r="G39">
-        <v>32.5</v>
+        <v>33.61</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
@@ -1639,13 +1642,13 @@
         <v>3</v>
       </c>
       <c r="E40">
-        <v>-8.99</v>
+        <v>-8.1999999999999993</v>
       </c>
       <c r="F40">
-        <v>5.01</v>
+        <v>5.91</v>
       </c>
       <c r="G40">
-        <v>25.14</v>
+        <v>26.22</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
@@ -1662,13 +1665,13 @@
         <v>2</v>
       </c>
       <c r="E41">
-        <v>-27.3</v>
+        <v>-29.25</v>
       </c>
       <c r="F41">
-        <v>3.55</v>
+        <v>0.95</v>
       </c>
       <c r="G41">
-        <v>32.979999999999997</v>
+        <v>29.42</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
@@ -1685,13 +1688,13 @@
         <v>0</v>
       </c>
       <c r="E42">
-        <v>-3.49</v>
+        <v>-0.64</v>
       </c>
       <c r="F42">
-        <v>11.05</v>
+        <v>14.33</v>
       </c>
       <c r="G42">
-        <v>27.65</v>
+        <v>31.41</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
@@ -1708,13 +1711,13 @@
         <v>1</v>
       </c>
       <c r="E43">
-        <v>-37.81</v>
+        <v>-39.33</v>
       </c>
       <c r="F43">
-        <v>4.62</v>
+        <v>2.89</v>
       </c>
       <c r="G43">
-        <v>31.15</v>
+        <v>27.93</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
@@ -1731,7 +1734,7 @@
         <v>1</v>
       </c>
       <c r="F44">
-        <v>-9.18</v>
+        <v>-7.58</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
@@ -1748,7 +1751,7 @@
         <v>0</v>
       </c>
       <c r="F45">
-        <v>32.65</v>
+        <v>30.65</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
@@ -1765,13 +1768,13 @@
         <v>0</v>
       </c>
       <c r="E46">
-        <v>4.96</v>
+        <v>6.18</v>
       </c>
       <c r="F46">
-        <v>7.82</v>
+        <v>9.07</v>
       </c>
       <c r="G46">
-        <v>10.69</v>
+        <v>11.97</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
@@ -1788,7 +1791,7 @@
         <v>1</v>
       </c>
       <c r="F47">
-        <v>-24.57</v>
+        <v>-21.57</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
@@ -1805,13 +1808,13 @@
         <v>2</v>
       </c>
       <c r="E48">
-        <v>-24.2</v>
+        <v>-23.93</v>
       </c>
       <c r="F48">
-        <v>-4.96</v>
+        <v>-4.62</v>
       </c>
       <c r="G48">
-        <v>16.62</v>
+        <v>17.03</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
@@ -1828,13 +1831,13 @@
         <v>0</v>
       </c>
       <c r="E49">
-        <v>9.23</v>
+        <v>6.77</v>
       </c>
       <c r="F49">
-        <v>12.31</v>
+        <v>9.77</v>
       </c>
       <c r="G49">
-        <v>15.38</v>
+        <v>12.78</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
@@ -1851,7 +1854,7 @@
         <v>0</v>
       </c>
       <c r="F50">
-        <v>3.31</v>
+        <v>1.1299999999999999</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
@@ -1868,7 +1871,7 @@
         <v>0</v>
       </c>
       <c r="F51">
-        <v>10.6</v>
+        <v>12.68</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
@@ -1876,16 +1879,13 @@
         <v>57</v>
       </c>
       <c r="B52">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C52">
         <v>0</v>
       </c>
       <c r="D52">
         <v>0</v>
-      </c>
-      <c r="F52">
-        <v>494.06</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
@@ -1902,7 +1902,7 @@
         <v>0</v>
       </c>
       <c r="F53">
-        <v>52.51</v>
+        <v>55.56</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
@@ -1935,9 +1935,6 @@
       <c r="D55">
         <v>1</v>
       </c>
-      <c r="F55">
-        <v>-1.2</v>
-      </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
@@ -1953,13 +1950,13 @@
         <v>2</v>
       </c>
       <c r="E56">
-        <v>-5.41</v>
+        <v>-4.4400000000000004</v>
       </c>
       <c r="F56">
-        <v>-4.46</v>
+        <v>-3.48</v>
       </c>
       <c r="G56">
-        <v>-2.7</v>
+        <v>-1.71</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
@@ -1976,13 +1973,13 @@
         <v>0</v>
       </c>
       <c r="E57">
-        <v>-0.47</v>
+        <v>-11.63</v>
       </c>
       <c r="F57">
-        <v>3.98</v>
+        <v>0.06</v>
       </c>
       <c r="G57">
-        <v>10.07</v>
+        <v>8.32</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.2">
@@ -1999,13 +1996,13 @@
         <v>1</v>
       </c>
       <c r="E58">
-        <v>2.48</v>
+        <v>2.0099999999999998</v>
       </c>
       <c r="F58">
-        <v>9.4700000000000006</v>
+        <v>8.9600000000000009</v>
       </c>
       <c r="G58">
-        <v>24.22</v>
+        <v>23.65</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
@@ -2022,13 +2019,13 @@
         <v>0</v>
       </c>
       <c r="E59">
-        <v>10.43</v>
+        <v>8.83</v>
       </c>
       <c r="F59">
-        <v>15.34</v>
+        <v>13.66</v>
       </c>
       <c r="G59">
-        <v>19.63</v>
+        <v>17.899999999999999</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.2">
@@ -2045,13 +2042,13 @@
         <v>1</v>
       </c>
       <c r="E60">
-        <v>-10.76</v>
+        <v>-10.34</v>
       </c>
       <c r="F60">
-        <v>0.37</v>
+        <v>0.83</v>
       </c>
       <c r="G60">
-        <v>9.84</v>
+        <v>10.34</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.2">
@@ -2068,13 +2065,13 @@
         <v>0</v>
       </c>
       <c r="E61">
-        <v>13.07</v>
+        <v>20</v>
       </c>
       <c r="F61">
-        <v>15.2</v>
+        <v>22.27</v>
       </c>
       <c r="G61">
-        <v>18.09</v>
+        <v>25.33</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.2">
@@ -2091,13 +2088,13 @@
         <v>3</v>
       </c>
       <c r="E62">
-        <v>-29.03</v>
+        <v>-28.76</v>
       </c>
       <c r="F62">
-        <v>-11.61</v>
+        <v>-11.27</v>
       </c>
       <c r="G62">
-        <v>-3.23</v>
+        <v>-2.85</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.2">
@@ -2114,13 +2111,13 @@
         <v>1</v>
       </c>
       <c r="E63">
-        <v>-3.8</v>
+        <v>-4.12</v>
       </c>
       <c r="F63">
-        <v>8.34</v>
+        <v>7.98</v>
       </c>
       <c r="G63">
-        <v>16.329999999999998</v>
+        <v>15.94</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.2">
@@ -2151,7 +2148,7 @@
         <v>0</v>
       </c>
       <c r="F65">
-        <v>16.600000000000001</v>
+        <v>17.079999999999998</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.2">
@@ -2191,13 +2188,13 @@
         <v>0</v>
       </c>
       <c r="E67">
-        <v>-19.399999999999999</v>
+        <v>-21.85</v>
       </c>
       <c r="F67">
-        <v>-11.64</v>
+        <v>-14.33</v>
       </c>
       <c r="G67">
-        <v>-4.4800000000000004</v>
+        <v>-7.38</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.2">
@@ -2228,13 +2225,13 @@
         <v>0</v>
       </c>
       <c r="E69">
-        <v>22.74</v>
+        <v>21.43</v>
       </c>
       <c r="F69">
-        <v>36.28</v>
+        <v>34.82</v>
       </c>
       <c r="G69">
-        <v>49.82</v>
+        <v>48.21</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.2">
@@ -2251,13 +2248,13 @@
         <v>0</v>
       </c>
       <c r="E70">
-        <v>7.64</v>
+        <v>8.93</v>
       </c>
       <c r="F70">
-        <v>11.25</v>
+        <v>12.58</v>
       </c>
       <c r="G70">
-        <v>13.02</v>
+        <v>14.38</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.2">
@@ -2274,7 +2271,7 @@
         <v>0</v>
       </c>
       <c r="F71">
-        <v>6.26</v>
+        <v>7.14</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.2">
@@ -2291,13 +2288,13 @@
         <v>0</v>
       </c>
       <c r="E72">
-        <v>-6.35</v>
+        <v>-4.22</v>
       </c>
       <c r="F72">
-        <v>8.73</v>
+        <v>11.2</v>
       </c>
       <c r="G72">
-        <v>19.05</v>
+        <v>21.75</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.2">
@@ -2314,13 +2311,13 @@
         <v>4</v>
       </c>
       <c r="E73">
-        <v>-39.25</v>
+        <v>-37.85</v>
       </c>
       <c r="F73">
-        <v>-17.5</v>
+        <v>-15.6</v>
       </c>
       <c r="G73">
-        <v>9.36</v>
+        <v>11.87</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.2">
@@ -2337,13 +2334,13 @@
         <v>2</v>
       </c>
       <c r="E74">
-        <v>-17.739999999999998</v>
+        <v>-15.57</v>
       </c>
       <c r="F74">
-        <v>-9.66</v>
+        <v>-7.27</v>
       </c>
       <c r="G74">
-        <v>0.14000000000000001</v>
+        <v>2.79</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.2">
@@ -2360,13 +2357,13 @@
         <v>0</v>
       </c>
       <c r="E75">
-        <v>14.7</v>
+        <v>18.03</v>
       </c>
       <c r="F75">
-        <v>22.52</v>
+        <v>26.07</v>
       </c>
       <c r="G75">
-        <v>30.34</v>
+        <v>34.119999999999997</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.2">
@@ -2397,7 +2394,7 @@
         <v>0</v>
       </c>
       <c r="F77">
-        <v>9.14</v>
+        <v>11.42</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.2">
@@ -2414,13 +2411,13 @@
         <v>1</v>
       </c>
       <c r="E78">
-        <v>-2.14</v>
+        <v>-0.93</v>
       </c>
       <c r="F78">
-        <v>10.09</v>
+        <v>11.46</v>
       </c>
       <c r="G78">
-        <v>22.32</v>
+        <v>23.84</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.2">
@@ -2437,13 +2434,13 @@
         <v>0</v>
       </c>
       <c r="E79">
-        <v>9.98</v>
+        <v>9.76</v>
       </c>
       <c r="F79">
-        <v>24.64</v>
+        <v>24.39</v>
       </c>
       <c r="G79">
-        <v>46.64</v>
+        <v>46.34</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.2">
@@ -2460,13 +2457,13 @@
         <v>1</v>
       </c>
       <c r="E80">
-        <v>2.83</v>
+        <v>4.58</v>
       </c>
       <c r="F80">
-        <v>10.029999999999999</v>
+        <v>11.9</v>
       </c>
       <c r="G80">
-        <v>15.68</v>
+        <v>17.649999999999999</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.2">
@@ -2483,13 +2480,13 @@
         <v>0</v>
       </c>
       <c r="E81">
-        <v>15.63</v>
+        <v>12.9</v>
       </c>
       <c r="F81">
-        <v>18.170000000000002</v>
+        <v>15.38</v>
       </c>
       <c r="G81">
-        <v>20.71</v>
+        <v>17.87</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.2">
@@ -2506,7 +2503,7 @@
         <v>1</v>
       </c>
       <c r="F82">
-        <v>-9.09</v>
+        <v>-10.57</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.2">
@@ -2523,13 +2520,13 @@
         <v>0</v>
       </c>
       <c r="E83">
-        <v>17.649999999999999</v>
+        <v>18.47</v>
       </c>
       <c r="F83">
-        <v>38.409999999999997</v>
+        <v>39.369999999999997</v>
       </c>
       <c r="G83">
-        <v>73.010000000000005</v>
+        <v>74.22</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.2">
@@ -2546,13 +2543,13 @@
         <v>0</v>
       </c>
       <c r="E84">
-        <v>2.8</v>
+        <v>2.91</v>
       </c>
       <c r="F84">
-        <v>22.95</v>
+        <v>23.08</v>
       </c>
       <c r="G84">
-        <v>45.38</v>
+        <v>45.53</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.2">
@@ -2569,13 +2566,13 @@
         <v>4</v>
       </c>
       <c r="E85">
-        <v>-19.75</v>
+        <v>-21.43</v>
       </c>
       <c r="F85">
-        <v>-11.28</v>
+        <v>-13.14</v>
       </c>
       <c r="G85">
-        <v>4.7699999999999996</v>
+        <v>2.58</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.2">
@@ -2592,7 +2589,7 @@
         <v>1</v>
       </c>
       <c r="F86">
-        <v>2.27</v>
+        <v>1.1200000000000001</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.2">
@@ -2609,7 +2606,7 @@
         <v>1</v>
       </c>
       <c r="F87">
-        <v>-11.76</v>
+        <v>-13.22</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.2">
@@ -2626,7 +2623,7 @@
         <v>1</v>
       </c>
       <c r="F88">
-        <v>-3.11</v>
+        <v>-0.71</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.2">
@@ -2643,13 +2640,13 @@
         <v>0</v>
       </c>
       <c r="E89">
-        <v>8.25</v>
+        <v>6.01</v>
       </c>
       <c r="F89">
-        <v>17.91</v>
+        <v>15.47</v>
       </c>
       <c r="G89">
-        <v>41.75</v>
+        <v>38.82</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.2">
@@ -2666,13 +2663,13 @@
         <v>0</v>
       </c>
       <c r="E90">
-        <v>10.87</v>
+        <v>10.47</v>
       </c>
       <c r="F90">
-        <v>15.07</v>
+        <v>14.66</v>
       </c>
       <c r="G90">
-        <v>19.57</v>
+        <v>19.13</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.2">
@@ -2689,7 +2686,7 @@
         <v>1</v>
       </c>
       <c r="F91">
-        <v>-9.2200000000000006</v>
+        <v>-5.12</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.2">
@@ -2706,7 +2703,7 @@
         <v>0</v>
       </c>
       <c r="F92">
-        <v>6.01</v>
+        <v>2.39</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.2">
@@ -2723,7 +2720,7 @@
         <v>0</v>
       </c>
       <c r="F93">
-        <v>-17.649999999999999</v>
+        <v>-15.05</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.2">
@@ -2740,7 +2737,7 @@
         <v>0</v>
       </c>
       <c r="F94">
-        <v>16.28</v>
+        <v>17.649999999999999</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.2">
@@ -2757,7 +2754,7 @@
         <v>2</v>
       </c>
       <c r="F95">
-        <v>16.670000000000002</v>
+        <v>18.64</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.2">
@@ -2774,13 +2771,13 @@
         <v>0</v>
       </c>
       <c r="E96">
-        <v>8.23</v>
+        <v>10.62</v>
       </c>
       <c r="F96">
-        <v>10.39</v>
+        <v>12.83</v>
       </c>
       <c r="G96">
-        <v>12.55</v>
+        <v>15.04</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.2">
@@ -2797,7 +2794,7 @@
         <v>1</v>
       </c>
       <c r="F97">
-        <v>4.05</v>
+        <v>2.86</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.2">
@@ -2814,13 +2811,13 @@
         <v>1</v>
       </c>
       <c r="E98">
-        <v>-5.31</v>
+        <v>-4.43</v>
       </c>
       <c r="F98">
-        <v>-0.69</v>
+        <v>0.23</v>
       </c>
       <c r="G98">
-        <v>5.08</v>
+        <v>6.06</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.2">
@@ -2837,13 +2834,13 @@
         <v>0</v>
       </c>
       <c r="E99">
-        <v>54.19</v>
+        <v>75.88</v>
       </c>
       <c r="F99">
-        <v>622.47</v>
+        <v>724.12</v>
       </c>
       <c r="G99">
-        <v>2468.2800000000002</v>
+        <v>2829.65</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.2">
@@ -2851,7 +2848,7 @@
         <v>105</v>
       </c>
       <c r="B100">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C100">
         <v>0</v>
@@ -2859,8 +2856,14 @@
       <c r="D100">
         <v>0</v>
       </c>
+      <c r="E100">
+        <v>5.36</v>
+      </c>
       <c r="F100">
-        <v>16.53</v>
+        <v>10.15</v>
+      </c>
+      <c r="G100">
+        <v>14.94</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.2">
@@ -2877,7 +2880,7 @@
         <v>1</v>
       </c>
       <c r="F101">
-        <v>-10.71</v>
+        <v>-16.670000000000002</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.2">
@@ -2894,7 +2897,7 @@
         <v>0</v>
       </c>
       <c r="F102">
-        <v>28.91</v>
+        <v>33.6</v>
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.2">
@@ -2911,13 +2914,13 @@
         <v>0</v>
       </c>
       <c r="E103">
-        <v>100.2</v>
+        <v>121.24</v>
       </c>
       <c r="F103">
-        <v>117.22</v>
+        <v>140.04</v>
       </c>
       <c r="G103">
-        <v>125.23</v>
+        <v>148.88999999999999</v>
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.2">
@@ -2934,13 +2937,13 @@
         <v>1</v>
       </c>
       <c r="E104">
-        <v>-13.53</v>
+        <v>-11</v>
       </c>
       <c r="F104">
-        <v>22.67</v>
+        <v>26.26</v>
       </c>
       <c r="G104">
-        <v>48.24</v>
+        <v>52.57</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.2">
@@ -2957,7 +2960,7 @@
         <v>0</v>
       </c>
       <c r="F105">
-        <v>15.38</v>
+        <v>18.71</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.2">
@@ -2974,13 +2977,13 @@
         <v>0</v>
       </c>
       <c r="E106">
-        <v>30.43</v>
+        <v>39</v>
       </c>
       <c r="F106">
-        <v>52.83</v>
+        <v>62.86</v>
       </c>
       <c r="G106">
-        <v>98.19</v>
+        <v>111.2</v>
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.2">
@@ -2997,7 +3000,7 @@
         <v>2</v>
       </c>
       <c r="F107">
-        <v>-20.69</v>
+        <v>-21.77</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.2">
@@ -3014,13 +3017,13 @@
         <v>1</v>
       </c>
       <c r="E108">
-        <v>6.38</v>
+        <v>-28.84</v>
       </c>
       <c r="F108">
-        <v>31.58</v>
+        <v>-11.99</v>
       </c>
       <c r="G108">
-        <v>56.77</v>
+        <v>4.87</v>
       </c>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.2">
@@ -3037,13 +3040,13 @@
         <v>0</v>
       </c>
       <c r="E109">
-        <v>7.05</v>
+        <v>9.25</v>
       </c>
       <c r="F109">
-        <v>15.24</v>
+        <v>17.61</v>
       </c>
       <c r="G109">
-        <v>25.94</v>
+        <v>28.53</v>
       </c>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.2">
@@ -3060,13 +3063,13 @@
         <v>0</v>
       </c>
       <c r="E110">
-        <v>-12</v>
+        <v>-8.14</v>
       </c>
       <c r="F110">
-        <v>4</v>
+        <v>8.56</v>
       </c>
       <c r="G110">
-        <v>20</v>
+        <v>25.26</v>
       </c>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.2">
@@ -3083,7 +3086,7 @@
         <v>1</v>
       </c>
       <c r="F111">
-        <v>23.42</v>
+        <v>27.45</v>
       </c>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.2">
@@ -3114,7 +3117,7 @@
         <v>0</v>
       </c>
       <c r="F113">
-        <v>15.23</v>
+        <v>14.75</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.2">
@@ -3131,13 +3134,13 @@
         <v>1</v>
       </c>
       <c r="E114">
-        <v>6.38</v>
+        <v>2.56</v>
       </c>
       <c r="F114">
-        <v>16.05</v>
+        <v>7.69</v>
       </c>
       <c r="G114">
-        <v>25.73</v>
+        <v>12.82</v>
       </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.2">
@@ -3154,13 +3157,13 @@
         <v>2</v>
       </c>
       <c r="E115">
-        <v>5.77</v>
+        <v>4.76</v>
       </c>
       <c r="F115">
-        <v>34.619999999999997</v>
+        <v>33.33</v>
       </c>
       <c r="G115">
-        <v>92.31</v>
+        <v>90.48</v>
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.2">
@@ -3177,7 +3180,7 @@
         <v>0</v>
       </c>
       <c r="F116">
-        <v>-11.31</v>
+        <v>-8.73</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.2">
@@ -3185,7 +3188,7 @@
         <v>122</v>
       </c>
       <c r="B117">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C117">
         <v>1</v>
@@ -3194,13 +3197,30 @@
         <v>0</v>
       </c>
       <c r="E117">
-        <v>-6.78</v>
+        <v>-9.19</v>
       </c>
       <c r="F117">
-        <v>15.5</v>
+        <v>25.2</v>
       </c>
       <c r="G117">
-        <v>37.89</v>
+        <v>50.46</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A118" t="s">
+        <v>123</v>
+      </c>
+      <c r="B118">
+        <v>2</v>
+      </c>
+      <c r="C118">
+        <v>0</v>
+      </c>
+      <c r="D118">
+        <v>0</v>
+      </c>
+      <c r="F118">
+        <v>5.49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Manual Analyst Ratings spreadsheet
</commit_message>
<xml_diff>
--- a/Manual_Analyst_Ratings.xlsx
+++ b/Manual_Analyst_Ratings.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/casperkangas/Documents/VS Code/Personal Projects/nordnet-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F741D978-F166-3E46-9F53-0464244FDDCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2949E6D-3A43-A842-B974-6B188A0BE962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="18000" yWindow="780" windowWidth="18000" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
   </bookViews>
@@ -813,19 +813,19 @@
         <v>15</v>
       </c>
       <c r="C2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D2">
         <v>5</v>
       </c>
       <c r="E2">
-        <v>-21.7</v>
+        <v>-22.27</v>
       </c>
       <c r="F2">
-        <v>2.91</v>
+        <v>2.89</v>
       </c>
       <c r="G2">
-        <v>15.21</v>
+        <v>14.38</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -842,13 +842,13 @@
         <v>2</v>
       </c>
       <c r="E3">
-        <v>-12.02</v>
+        <v>-8.16</v>
       </c>
       <c r="F3">
-        <v>16.62</v>
+        <v>21.73</v>
       </c>
       <c r="G3">
-        <v>71.069999999999993</v>
+        <v>78.569999999999993</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -856,22 +856,22 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C4">
         <v>6</v>
       </c>
       <c r="D4">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E4">
-        <v>-49.35</v>
+        <v>-51.56</v>
       </c>
       <c r="F4">
-        <v>20.37</v>
+        <v>17.29</v>
       </c>
       <c r="G4">
-        <v>96.08</v>
+        <v>87.5</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -888,13 +888,13 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>-2.46</v>
+        <v>-4.08</v>
       </c>
       <c r="F5">
-        <v>0.38</v>
+        <v>-1.28</v>
       </c>
       <c r="G5">
-        <v>3.69</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -911,13 +911,13 @@
         <v>5</v>
       </c>
       <c r="E6">
-        <v>-20.51</v>
+        <v>-20.260000000000002</v>
       </c>
       <c r="F6">
-        <v>-2.7</v>
+        <v>-2.39</v>
       </c>
       <c r="G6">
-        <v>11.29</v>
+        <v>11.64</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -934,7 +934,7 @@
         <v>1</v>
       </c>
       <c r="F7">
-        <v>0.12</v>
+        <v>-0.7</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -951,13 +951,13 @@
         <v>1</v>
       </c>
       <c r="E8">
-        <v>-37</v>
+        <v>-33.53</v>
       </c>
       <c r="F8">
-        <v>-3.12</v>
+        <v>2.21</v>
       </c>
       <c r="G8">
-        <v>14.55</v>
+        <v>20.85</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -974,7 +974,7 @@
         <v>0</v>
       </c>
       <c r="F9">
-        <v>3.34</v>
+        <v>-1.22</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -991,13 +991,13 @@
         <v>3</v>
       </c>
       <c r="E10">
-        <v>-34.75</v>
+        <v>-34.479999999999997</v>
       </c>
       <c r="F10">
-        <v>14.87</v>
+        <v>15.72</v>
       </c>
       <c r="G10">
-        <v>47.55</v>
+        <v>48.28</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -1014,13 +1014,13 @@
         <v>1</v>
       </c>
       <c r="E11">
-        <v>-11.63</v>
+        <v>-11.17</v>
       </c>
       <c r="F11">
-        <v>20.38</v>
+        <v>21</v>
       </c>
       <c r="G11">
-        <v>63</v>
+        <v>63.84</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -1037,13 +1037,13 @@
         <v>3</v>
       </c>
       <c r="E12">
-        <v>-25.62</v>
+        <v>-22.19</v>
       </c>
       <c r="F12">
-        <v>-1.32</v>
+        <v>3.92</v>
       </c>
       <c r="G12">
-        <v>18.46</v>
+        <v>23.92</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -1051,7 +1051,7 @@
         <v>18</v>
       </c>
       <c r="B13">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C13">
         <v>6</v>
@@ -1060,13 +1060,13 @@
         <v>2</v>
       </c>
       <c r="E13">
-        <v>-43.7</v>
+        <v>-46.25</v>
       </c>
       <c r="F13">
-        <v>6.33</v>
+        <v>3.07</v>
       </c>
       <c r="G13">
-        <v>62.18</v>
+        <v>54.83</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -1074,22 +1074,22 @@
         <v>19</v>
       </c>
       <c r="B14">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C14">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D14">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E14">
-        <v>-31.16</v>
+        <v>-37.18</v>
       </c>
       <c r="F14">
-        <v>-14.14</v>
+        <v>-7.57</v>
       </c>
       <c r="G14">
-        <v>3.72</v>
+        <v>24.78</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -1106,13 +1106,13 @@
         <v>0</v>
       </c>
       <c r="E15">
-        <v>25.43</v>
+        <v>27.87</v>
       </c>
       <c r="F15">
-        <v>34.08</v>
+        <v>36.68</v>
       </c>
       <c r="G15">
-        <v>42.73</v>
+        <v>45.5</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -1129,13 +1129,13 @@
         <v>0</v>
       </c>
       <c r="E16">
-        <v>-1.1599999999999999</v>
+        <v>1.39</v>
       </c>
       <c r="F16">
-        <v>9.44</v>
+        <v>12.26</v>
       </c>
       <c r="G16">
-        <v>16.399999999999999</v>
+        <v>19.399999999999999</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
@@ -1152,13 +1152,13 @@
         <v>5</v>
       </c>
       <c r="E17">
-        <v>-27.86</v>
+        <v>-21.93</v>
       </c>
       <c r="F17">
-        <v>7.59</v>
+        <v>2.35</v>
       </c>
       <c r="G17">
-        <v>57.55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
@@ -1175,13 +1175,13 @@
         <v>2</v>
       </c>
       <c r="E18">
-        <v>-21.38</v>
+        <v>-14.89</v>
       </c>
       <c r="F18">
-        <v>9.8800000000000008</v>
+        <v>6.76</v>
       </c>
       <c r="G18">
-        <v>32.68</v>
+        <v>27.66</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
@@ -1198,13 +1198,13 @@
         <v>2</v>
       </c>
       <c r="E19">
-        <v>-30.82</v>
+        <v>-33.61</v>
       </c>
       <c r="F19">
-        <v>-2.6</v>
+        <v>-6.54</v>
       </c>
       <c r="G19">
-        <v>8.18</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
@@ -1221,13 +1221,13 @@
         <v>2</v>
       </c>
       <c r="E20">
-        <v>4.05</v>
+        <v>-3.87</v>
       </c>
       <c r="F20">
-        <v>13.93</v>
+        <v>5.26</v>
       </c>
       <c r="G20">
-        <v>24.28</v>
+        <v>14.82</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -1238,19 +1238,19 @@
         <v>7</v>
       </c>
       <c r="C21">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D21">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E21">
-        <v>-5.86</v>
+        <v>-10.89</v>
       </c>
       <c r="F21">
-        <v>10.6</v>
+        <v>4.1900000000000004</v>
       </c>
       <c r="G21">
-        <v>40.92</v>
+        <v>33.4</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -1264,16 +1264,16 @@
         <v>11</v>
       </c>
       <c r="D22">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E22">
-        <v>-30.5</v>
+        <v>-32.619999999999997</v>
       </c>
       <c r="F22">
-        <v>5</v>
+        <v>1.55</v>
       </c>
       <c r="G22">
-        <v>36</v>
+        <v>25.06</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
@@ -1284,19 +1284,19 @@
         <v>3</v>
       </c>
       <c r="C23">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D23">
         <v>1</v>
       </c>
       <c r="E23">
-        <v>-18.05</v>
+        <v>-16</v>
       </c>
       <c r="F23">
-        <v>-1.45</v>
+        <v>1.54</v>
       </c>
       <c r="G23">
-        <v>21.89</v>
+        <v>24.93</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
@@ -1313,13 +1313,13 @@
         <v>0</v>
       </c>
       <c r="E24">
-        <v>2.35</v>
+        <v>2.88</v>
       </c>
       <c r="F24">
-        <v>7.47</v>
+        <v>8.02</v>
       </c>
       <c r="G24">
-        <v>17.71</v>
+        <v>18.309999999999999</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
@@ -1336,13 +1336,13 @@
         <v>0</v>
       </c>
       <c r="E25">
-        <v>18.690000000000001</v>
+        <v>20.48</v>
       </c>
       <c r="F25">
-        <v>21.66</v>
+        <v>23.49</v>
       </c>
       <c r="G25">
-        <v>24.63</v>
+        <v>26.51</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
@@ -1359,7 +1359,7 @@
         <v>0</v>
       </c>
       <c r="F26">
-        <v>-15.25</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
@@ -1376,7 +1376,7 @@
         <v>0</v>
       </c>
       <c r="F27">
-        <v>6.25</v>
+        <v>13.33</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
@@ -1393,7 +1393,7 @@
         <v>1</v>
       </c>
       <c r="F28">
-        <v>10.97</v>
+        <v>21.78</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
@@ -1424,7 +1424,7 @@
         <v>0</v>
       </c>
       <c r="F30">
-        <v>11.11</v>
+        <v>10.66</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -1441,13 +1441,13 @@
         <v>2</v>
       </c>
       <c r="E31">
-        <v>7.14</v>
+        <v>8.84</v>
       </c>
       <c r="F31">
-        <v>9.3800000000000008</v>
+        <v>11.11</v>
       </c>
       <c r="G31">
-        <v>11.61</v>
+        <v>13.38</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
@@ -1464,13 +1464,13 @@
         <v>0</v>
       </c>
       <c r="E32">
-        <v>6.04</v>
+        <v>8.41</v>
       </c>
       <c r="F32">
-        <v>21.66</v>
+        <v>24.38</v>
       </c>
       <c r="G32">
-        <v>34.96</v>
+        <v>37.979999999999997</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
@@ -1487,7 +1487,7 @@
         <v>0</v>
       </c>
       <c r="F33">
-        <v>15.77</v>
+        <v>18.64</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
@@ -1504,13 +1504,13 @@
         <v>1</v>
       </c>
       <c r="E34">
-        <v>-1.81</v>
+        <v>-1.68</v>
       </c>
       <c r="F34">
-        <v>17.18</v>
+        <v>17.34</v>
       </c>
       <c r="G34">
-        <v>29.2</v>
+        <v>29.37</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
@@ -1527,13 +1527,13 @@
         <v>0</v>
       </c>
       <c r="E35">
-        <v>-1.1299999999999999</v>
+        <v>-5.75</v>
       </c>
       <c r="F35">
-        <v>16.95</v>
+        <v>11.49</v>
       </c>
       <c r="G35">
-        <v>31.83</v>
+        <v>25.67</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
@@ -1550,13 +1550,13 @@
         <v>0</v>
       </c>
       <c r="E36">
-        <v>10.6</v>
+        <v>4.42</v>
       </c>
       <c r="F36">
-        <v>27.55</v>
+        <v>25.46</v>
       </c>
       <c r="G36">
-        <v>43.05</v>
+        <v>44.82</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
@@ -1573,13 +1573,13 @@
         <v>0</v>
       </c>
       <c r="E37">
-        <v>7.78</v>
+        <v>10.73</v>
       </c>
       <c r="F37">
-        <v>10</v>
+        <v>13.01</v>
       </c>
       <c r="G37">
-        <v>11.11</v>
+        <v>14.16</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
@@ -1596,13 +1596,13 @@
         <v>0</v>
       </c>
       <c r="E38">
-        <v>5.01</v>
+        <v>6.09</v>
       </c>
       <c r="F38">
-        <v>17.579999999999998</v>
+        <v>18.79</v>
       </c>
       <c r="G38">
-        <v>28.73</v>
+        <v>30.05</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
@@ -1619,13 +1619,13 @@
         <v>0</v>
       </c>
       <c r="E39">
-        <v>-5.0599999999999996</v>
+        <v>-3.43</v>
       </c>
       <c r="F39">
-        <v>11.01</v>
+        <v>13.3</v>
       </c>
       <c r="G39">
-        <v>33.61</v>
+        <v>35.909999999999997</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
@@ -1642,13 +1642,13 @@
         <v>3</v>
       </c>
       <c r="E40">
-        <v>-8.1999999999999993</v>
+        <v>-7.08</v>
       </c>
       <c r="F40">
-        <v>5.91</v>
+        <v>7.2</v>
       </c>
       <c r="G40">
-        <v>26.22</v>
+        <v>27.76</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
@@ -1665,13 +1665,13 @@
         <v>2</v>
       </c>
       <c r="E41">
-        <v>-29.25</v>
+        <v>-21.98</v>
       </c>
       <c r="F41">
-        <v>0.95</v>
+        <v>11.89</v>
       </c>
       <c r="G41">
-        <v>29.42</v>
+        <v>42.72</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
@@ -1688,13 +1688,13 @@
         <v>0</v>
       </c>
       <c r="E42">
-        <v>-0.64</v>
+        <v>2.38</v>
       </c>
       <c r="F42">
-        <v>14.33</v>
+        <v>17.8</v>
       </c>
       <c r="G42">
-        <v>31.41</v>
+        <v>35.4</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
@@ -1711,13 +1711,13 @@
         <v>1</v>
       </c>
       <c r="E43">
-        <v>-39.33</v>
+        <v>-32.229999999999997</v>
       </c>
       <c r="F43">
-        <v>2.89</v>
+        <v>5.18</v>
       </c>
       <c r="G43">
-        <v>27.93</v>
+        <v>30.25</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
@@ -1734,7 +1734,7 @@
         <v>1</v>
       </c>
       <c r="F44">
-        <v>-7.58</v>
+        <v>-10.19</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
@@ -1751,7 +1751,7 @@
         <v>0</v>
       </c>
       <c r="F45">
-        <v>30.65</v>
+        <v>4.21</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
@@ -1768,13 +1768,13 @@
         <v>0</v>
       </c>
       <c r="E46">
-        <v>6.18</v>
+        <v>-2.83</v>
       </c>
       <c r="F46">
-        <v>9.07</v>
+        <v>-0.18</v>
       </c>
       <c r="G46">
-        <v>11.97</v>
+        <v>2.4700000000000002</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
@@ -1791,7 +1791,7 @@
         <v>1</v>
       </c>
       <c r="F47">
-        <v>-21.57</v>
+        <v>-18</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
@@ -1808,13 +1808,13 @@
         <v>2</v>
       </c>
       <c r="E48">
-        <v>-23.93</v>
+        <v>-23.55</v>
       </c>
       <c r="F48">
-        <v>-4.62</v>
+        <v>-3.89</v>
       </c>
       <c r="G48">
-        <v>17.03</v>
+        <v>17.920000000000002</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
@@ -1831,13 +1831,13 @@
         <v>0</v>
       </c>
       <c r="E49">
-        <v>6.77</v>
+        <v>1.43</v>
       </c>
       <c r="F49">
-        <v>9.77</v>
+        <v>4.29</v>
       </c>
       <c r="G49">
-        <v>12.78</v>
+        <v>7.14</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
@@ -1854,7 +1854,7 @@
         <v>0</v>
       </c>
       <c r="F50">
-        <v>1.1299999999999999</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
@@ -1871,7 +1871,7 @@
         <v>0</v>
       </c>
       <c r="F51">
-        <v>12.68</v>
+        <v>20.72</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
@@ -1902,7 +1902,7 @@
         <v>0</v>
       </c>
       <c r="F53">
-        <v>55.56</v>
+        <v>26.44</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
@@ -1919,7 +1919,7 @@
         <v>0</v>
       </c>
       <c r="F54">
-        <v>25.55</v>
+        <v>27.78</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
@@ -1935,6 +1935,9 @@
       <c r="D55">
         <v>1</v>
       </c>
+      <c r="F55">
+        <v>11.49</v>
+      </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
@@ -1950,13 +1953,13 @@
         <v>2</v>
       </c>
       <c r="E56">
-        <v>-4.4400000000000004</v>
+        <v>-0.28000000000000003</v>
       </c>
       <c r="F56">
-        <v>-3.48</v>
+        <v>0.71</v>
       </c>
       <c r="G56">
-        <v>-1.71</v>
+        <v>2.56</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
@@ -1973,13 +1976,13 @@
         <v>0</v>
       </c>
       <c r="E57">
-        <v>-11.63</v>
+        <v>-11.43</v>
       </c>
       <c r="F57">
-        <v>0.06</v>
+        <v>3.83</v>
       </c>
       <c r="G57">
-        <v>8.32</v>
+        <v>14.29</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.2">
@@ -1996,13 +1999,13 @@
         <v>1</v>
       </c>
       <c r="E58">
-        <v>2.0099999999999998</v>
+        <v>1.23</v>
       </c>
       <c r="F58">
-        <v>8.9600000000000009</v>
+        <v>8.1300000000000008</v>
       </c>
       <c r="G58">
-        <v>23.65</v>
+        <v>22.7</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
@@ -2019,13 +2022,13 @@
         <v>0</v>
       </c>
       <c r="E59">
-        <v>8.83</v>
+        <v>4.6500000000000004</v>
       </c>
       <c r="F59">
-        <v>13.66</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="G59">
-        <v>17.899999999999999</v>
+        <v>13.37</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.2">
@@ -2042,13 +2045,13 @@
         <v>1</v>
       </c>
       <c r="E60">
-        <v>-10.34</v>
+        <v>-10.76</v>
       </c>
       <c r="F60">
-        <v>0.83</v>
+        <v>1.65</v>
       </c>
       <c r="G60">
-        <v>10.34</v>
+        <v>12.13</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.2">
@@ -2065,13 +2068,13 @@
         <v>0</v>
       </c>
       <c r="E61">
-        <v>20</v>
+        <v>17.8</v>
       </c>
       <c r="F61">
-        <v>22.27</v>
+        <v>20.03</v>
       </c>
       <c r="G61">
-        <v>25.33</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.2">
@@ -2088,13 +2091,13 @@
         <v>3</v>
       </c>
       <c r="E62">
-        <v>-28.76</v>
+        <v>-27.15</v>
       </c>
       <c r="F62">
-        <v>-11.27</v>
+        <v>-9.27</v>
       </c>
       <c r="G62">
-        <v>-2.85</v>
+        <v>-0.66</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.2">
@@ -2111,13 +2114,13 @@
         <v>1</v>
       </c>
       <c r="E63">
-        <v>-4.12</v>
+        <v>0.47</v>
       </c>
       <c r="F63">
-        <v>7.98</v>
+        <v>13.15</v>
       </c>
       <c r="G63">
-        <v>15.94</v>
+        <v>21.5</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.2">
@@ -2148,7 +2151,7 @@
         <v>0</v>
       </c>
       <c r="F65">
-        <v>17.079999999999998</v>
+        <v>17.239999999999998</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.2">
@@ -2165,13 +2168,13 @@
         <v>1</v>
       </c>
       <c r="E66">
-        <v>-3.36</v>
+        <v>-6.5</v>
       </c>
       <c r="F66">
-        <v>11.34</v>
+        <v>7.72</v>
       </c>
       <c r="G66">
-        <v>38.659999999999997</v>
+        <v>34.15</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.2">
@@ -2188,13 +2191,13 @@
         <v>0</v>
       </c>
       <c r="E67">
-        <v>-21.85</v>
+        <v>-28.57</v>
       </c>
       <c r="F67">
-        <v>-14.33</v>
+        <v>-21.69</v>
       </c>
       <c r="G67">
-        <v>-7.38</v>
+        <v>-15.34</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.2">
@@ -2208,7 +2211,7 @@
         <v>0</v>
       </c>
       <c r="D68">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.2">
@@ -2248,13 +2251,13 @@
         <v>0</v>
       </c>
       <c r="E70">
-        <v>8.93</v>
+        <v>9.0500000000000007</v>
       </c>
       <c r="F70">
-        <v>12.58</v>
+        <v>12.7</v>
       </c>
       <c r="G70">
-        <v>14.38</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.2">
@@ -2271,7 +2274,7 @@
         <v>0</v>
       </c>
       <c r="F71">
-        <v>7.14</v>
+        <v>15.85</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.2">
@@ -2279,22 +2282,22 @@
         <v>77</v>
       </c>
       <c r="B72">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C72">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D72">
         <v>0</v>
       </c>
       <c r="E72">
-        <v>-4.22</v>
+        <v>3.01</v>
       </c>
       <c r="F72">
-        <v>11.2</v>
+        <v>11.33</v>
       </c>
       <c r="G72">
-        <v>21.75</v>
+        <v>18.86</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.2">
@@ -2311,13 +2314,13 @@
         <v>4</v>
       </c>
       <c r="E73">
-        <v>-37.85</v>
+        <v>-37.54</v>
       </c>
       <c r="F73">
-        <v>-15.6</v>
+        <v>-15.18</v>
       </c>
       <c r="G73">
-        <v>11.87</v>
+        <v>12.43</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.2">
@@ -2334,13 +2337,13 @@
         <v>2</v>
       </c>
       <c r="E74">
-        <v>-15.57</v>
+        <v>-12.61</v>
       </c>
       <c r="F74">
-        <v>-7.27</v>
+        <v>-4.03</v>
       </c>
       <c r="G74">
-        <v>2.79</v>
+        <v>6.38</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.2">
@@ -2357,13 +2360,13 @@
         <v>0</v>
       </c>
       <c r="E75">
-        <v>18.03</v>
+        <v>14.7</v>
       </c>
       <c r="F75">
-        <v>26.07</v>
+        <v>22.52</v>
       </c>
       <c r="G75">
-        <v>34.119999999999997</v>
+        <v>30.34</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.2">
@@ -2394,7 +2397,7 @@
         <v>0</v>
       </c>
       <c r="F77">
-        <v>11.42</v>
+        <v>13.31</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.2">
@@ -2411,13 +2414,13 @@
         <v>1</v>
       </c>
       <c r="E78">
-        <v>-0.93</v>
+        <v>-5.88</v>
       </c>
       <c r="F78">
-        <v>11.46</v>
+        <v>5.88</v>
       </c>
       <c r="G78">
-        <v>23.84</v>
+        <v>17.649999999999999</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.2">
@@ -2425,22 +2428,22 @@
         <v>84</v>
       </c>
       <c r="B79">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C79">
         <v>0</v>
       </c>
       <c r="D79">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E79">
-        <v>9.76</v>
+        <v>8.4600000000000009</v>
       </c>
       <c r="F79">
-        <v>24.39</v>
+        <v>31.02</v>
       </c>
       <c r="G79">
-        <v>46.34</v>
+        <v>56.18</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.2">
@@ -2457,13 +2460,13 @@
         <v>1</v>
       </c>
       <c r="E80">
-        <v>4.58</v>
+        <v>1.91</v>
       </c>
       <c r="F80">
-        <v>11.9</v>
+        <v>9.0399999999999991</v>
       </c>
       <c r="G80">
-        <v>17.649999999999999</v>
+        <v>14.65</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.2">
@@ -2480,13 +2483,13 @@
         <v>0</v>
       </c>
       <c r="E81">
-        <v>12.9</v>
+        <v>10.71</v>
       </c>
       <c r="F81">
-        <v>15.38</v>
+        <v>13.14</v>
       </c>
       <c r="G81">
-        <v>17.87</v>
+        <v>15.57</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.2">
@@ -2503,7 +2506,7 @@
         <v>1</v>
       </c>
       <c r="F82">
-        <v>-10.57</v>
+        <v>-15.38</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.2">
@@ -2520,13 +2523,13 @@
         <v>0</v>
       </c>
       <c r="E83">
-        <v>18.47</v>
+        <v>20.14</v>
       </c>
       <c r="F83">
-        <v>39.369999999999997</v>
+        <v>41.34</v>
       </c>
       <c r="G83">
-        <v>74.22</v>
+        <v>76.680000000000007</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.2">
@@ -2543,13 +2546,13 @@
         <v>0</v>
       </c>
       <c r="E84">
-        <v>2.91</v>
+        <v>2.27</v>
       </c>
       <c r="F84">
-        <v>23.08</v>
+        <v>22.31</v>
       </c>
       <c r="G84">
-        <v>45.53</v>
+        <v>44.63</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.2">
@@ -2566,13 +2569,13 @@
         <v>4</v>
       </c>
       <c r="E85">
-        <v>-21.43</v>
+        <v>-20.420000000000002</v>
       </c>
       <c r="F85">
-        <v>-13.14</v>
+        <v>-12.02</v>
       </c>
       <c r="G85">
-        <v>2.58</v>
+        <v>3.89</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.2">
@@ -2589,7 +2592,7 @@
         <v>1</v>
       </c>
       <c r="F86">
-        <v>1.1200000000000001</v>
+        <v>2.97</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.2">
@@ -2606,7 +2609,7 @@
         <v>1</v>
       </c>
       <c r="F87">
-        <v>-13.22</v>
+        <v>-15.32</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.2">
@@ -2623,7 +2626,7 @@
         <v>1</v>
       </c>
       <c r="F88">
-        <v>-0.71</v>
+        <v>-2.78</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.2">
@@ -2640,13 +2643,13 @@
         <v>0</v>
       </c>
       <c r="E89">
-        <v>6.01</v>
+        <v>7.91</v>
       </c>
       <c r="F89">
-        <v>15.47</v>
+        <v>17.55</v>
       </c>
       <c r="G89">
-        <v>38.82</v>
+        <v>41.32</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.2">
@@ -2663,13 +2666,13 @@
         <v>0</v>
       </c>
       <c r="E90">
-        <v>10.47</v>
+        <v>11.68</v>
       </c>
       <c r="F90">
-        <v>14.66</v>
+        <v>15.91</v>
       </c>
       <c r="G90">
-        <v>19.13</v>
+        <v>20.440000000000001</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.2">
@@ -2686,7 +2689,7 @@
         <v>1</v>
       </c>
       <c r="F91">
-        <v>-5.12</v>
+        <v>6.78</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.2">
@@ -2703,7 +2706,7 @@
         <v>0</v>
       </c>
       <c r="F92">
-        <v>2.39</v>
+        <v>-6.25</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.2">
@@ -2720,7 +2723,7 @@
         <v>0</v>
       </c>
       <c r="F93">
-        <v>-15.05</v>
+        <v>-23.58</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.2">
@@ -2737,7 +2740,7 @@
         <v>0</v>
       </c>
       <c r="F94">
-        <v>17.649999999999999</v>
+        <v>10.29</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.2">
@@ -2754,7 +2757,7 @@
         <v>2</v>
       </c>
       <c r="F95">
-        <v>18.64</v>
+        <v>17.45</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.2">
@@ -2771,13 +2774,13 @@
         <v>0</v>
       </c>
       <c r="E96">
-        <v>10.62</v>
+        <v>2.04</v>
       </c>
       <c r="F96">
-        <v>12.83</v>
+        <v>4.08</v>
       </c>
       <c r="G96">
-        <v>15.04</v>
+        <v>6.12</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.2">
@@ -2794,7 +2797,7 @@
         <v>1</v>
       </c>
       <c r="F97">
-        <v>2.86</v>
+        <v>-8.16</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.2">
@@ -2811,13 +2814,13 @@
         <v>1</v>
       </c>
       <c r="E98">
-        <v>-4.43</v>
+        <v>-1.2</v>
       </c>
       <c r="F98">
-        <v>0.23</v>
+        <v>3.61</v>
       </c>
       <c r="G98">
-        <v>6.06</v>
+        <v>9.64</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.2">
@@ -2834,13 +2837,13 @@
         <v>0</v>
       </c>
       <c r="E99">
-        <v>75.88</v>
+        <v>72.41</v>
       </c>
       <c r="F99">
-        <v>724.12</v>
+        <v>707.88</v>
       </c>
       <c r="G99">
-        <v>2829.65</v>
+        <v>2771.92</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.2">
@@ -2857,13 +2860,13 @@
         <v>0</v>
       </c>
       <c r="E100">
-        <v>5.36</v>
+        <v>13.4</v>
       </c>
       <c r="F100">
-        <v>10.15</v>
+        <v>18.559999999999999</v>
       </c>
       <c r="G100">
-        <v>14.94</v>
+        <v>23.71</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.2">
@@ -2880,7 +2883,7 @@
         <v>1</v>
       </c>
       <c r="F101">
-        <v>-16.670000000000002</v>
+        <v>-27.01</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.2">
@@ -2897,7 +2900,7 @@
         <v>0</v>
       </c>
       <c r="F102">
-        <v>33.6</v>
+        <v>35.25</v>
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.2">
@@ -2914,13 +2917,13 @@
         <v>0</v>
       </c>
       <c r="E103">
-        <v>121.24</v>
+        <v>124.97</v>
       </c>
       <c r="F103">
-        <v>140.04</v>
+        <v>144.09</v>
       </c>
       <c r="G103">
-        <v>148.88999999999999</v>
+        <v>153.09</v>
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.2">
@@ -2928,22 +2931,22 @@
         <v>109</v>
       </c>
       <c r="B104">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C104">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D104">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E104">
-        <v>-11</v>
+        <v>-6.85</v>
       </c>
       <c r="F104">
-        <v>26.26</v>
+        <v>30.54</v>
       </c>
       <c r="G104">
-        <v>52.57</v>
+        <v>59.68</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.2">
@@ -2960,7 +2963,7 @@
         <v>0</v>
       </c>
       <c r="F105">
-        <v>18.71</v>
+        <v>17.02</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.2">
@@ -2977,13 +2980,13 @@
         <v>0</v>
       </c>
       <c r="E106">
-        <v>39</v>
+        <v>35.85</v>
       </c>
       <c r="F106">
-        <v>62.86</v>
+        <v>64.42</v>
       </c>
       <c r="G106">
-        <v>111.2</v>
+        <v>106.42</v>
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.2">
@@ -3000,7 +3003,7 @@
         <v>2</v>
       </c>
       <c r="F107">
-        <v>-21.77</v>
+        <v>-24.59</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.2">
@@ -3017,13 +3020,13 @@
         <v>1</v>
       </c>
       <c r="E108">
-        <v>-28.84</v>
+        <v>-5.66</v>
       </c>
       <c r="F108">
-        <v>-11.99</v>
+        <v>13.21</v>
       </c>
       <c r="G108">
-        <v>4.87</v>
+        <v>32.08</v>
       </c>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.2">
@@ -3040,13 +3043,13 @@
         <v>0</v>
       </c>
       <c r="E109">
-        <v>9.25</v>
+        <v>12.43</v>
       </c>
       <c r="F109">
-        <v>17.61</v>
+        <v>21.03</v>
       </c>
       <c r="G109">
-        <v>28.53</v>
+        <v>32.28</v>
       </c>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.2">
@@ -3063,13 +3066,13 @@
         <v>0</v>
       </c>
       <c r="E110">
-        <v>-8.14</v>
+        <v>-2.2200000000000002</v>
       </c>
       <c r="F110">
-        <v>8.56</v>
+        <v>15.56</v>
       </c>
       <c r="G110">
-        <v>25.26</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.2">
@@ -3086,7 +3089,7 @@
         <v>1</v>
       </c>
       <c r="F111">
-        <v>27.45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.2">
@@ -3134,13 +3137,13 @@
         <v>1</v>
       </c>
       <c r="E114">
-        <v>2.56</v>
+        <v>10.130000000000001</v>
       </c>
       <c r="F114">
-        <v>7.69</v>
+        <v>15.64</v>
       </c>
       <c r="G114">
-        <v>12.82</v>
+        <v>21.15</v>
       </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.2">
@@ -3157,13 +3160,13 @@
         <v>2</v>
       </c>
       <c r="E115">
-        <v>4.76</v>
+        <v>1.85</v>
       </c>
       <c r="F115">
-        <v>33.33</v>
+        <v>29.63</v>
       </c>
       <c r="G115">
-        <v>90.48</v>
+        <v>85.19</v>
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.2">
@@ -3180,7 +3183,7 @@
         <v>0</v>
       </c>
       <c r="F116">
-        <v>-8.73</v>
+        <v>-4.96</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.2">
@@ -3197,13 +3200,13 @@
         <v>0</v>
       </c>
       <c r="E117">
-        <v>-9.19</v>
+        <v>-5.53</v>
       </c>
       <c r="F117">
-        <v>25.2</v>
+        <v>30.24</v>
       </c>
       <c r="G117">
-        <v>50.46</v>
+        <v>56.51</v>
       </c>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.2">
@@ -3220,7 +3223,7 @@
         <v>0</v>
       </c>
       <c r="F118">
-        <v>5.49</v>
+        <v>4.3499999999999996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>